<commit_message>
Fachada La Carreta: lenguaje claro (lados y puerta en vez de vano)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DFEggjd6XpHEYcqFvcrgyh
</commit_message>
<xml_diff>
--- a/fachada-la-carreta/lista-materiales-fachada-la-carreta.xlsx
+++ b/fachada-la-carreta/lista-materiales-fachada-la-carreta.xlsx
@@ -132,7 +132,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Un riel de 3,55 m (luz entre columnas) por vano con puertas</t>
+          <t xml:space="preserve">Un riel de 3,55 m (entre columnas) por puerta corrediza</t>
         </is>
       </c>
     </row>
@@ -152,7 +152,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Una guía de 3,55 m (luz entre columnas) por vano con puertas</t>
+          <t xml:space="preserve">Una guía de 3,55 m (entre columnas) por puerta corrediza</t>
         </is>
       </c>
     </row>
@@ -242,7 +242,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sobre el cierre central de cada vano</t>
+          <t xml:space="preserve">Sobre el cierre central de la puerta</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fachada La Carreta: los 4 lados con la misma luz entre columnas y opciones de puerta simples
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DFEggjd6XpHEYcqFvcrgyh
</commit_message>
<xml_diff>
--- a/fachada-la-carreta/lista-materiales-fachada-la-carreta.xlsx
+++ b/fachada-la-carreta/lista-materiales-fachada-la-carreta.xlsx
@@ -103,7 +103,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -112,7 +112,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">sobrante 14,16 m</t>
+          <t xml:space="preserve">sobrante 13,02 m</t>
         </is>
       </c>
     </row>
@@ -317,7 +317,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Área de tubo: 27,1 m², una mano</t>
+          <t xml:space="preserve">Área de tubo: 28,2 m², una mano</t>
         </is>
       </c>
     </row>
@@ -357,7 +357,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mi cálculo para 450 uniones soldadas. Con las medidas anteriores usaste 3 lb</t>
+          <t xml:space="preserve">Mi cálculo para 466 uniones soldadas. Con las medidas anteriores usaste 3 lb</t>
         </is>
       </c>
     </row>
@@ -418,7 +418,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C3">
@@ -431,7 +431,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C4">
@@ -444,7 +444,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C5">
@@ -457,11 +457,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,325 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C6">
-        <v>0.31</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="7">
@@ -470,11 +470,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,325 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C7">
-        <v>0.31</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="8">
@@ -483,11 +483,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,325 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C8">
-        <v>0.31</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="9">
@@ -496,11 +496,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,325 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C9">
-        <v>0.31</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="10">
@@ -509,11 +509,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,325 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C10">
-        <v>0.31</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="11">
@@ -522,11 +522,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,325 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C11">
-        <v>0.31</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="12">
@@ -743,7 +743,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,470 m (Der) + 1 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C28">
@@ -756,7 +756,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">3 × 1,470 m (Der) + 1 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C29">
@@ -899,7 +899,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,470 m (Izq) + 1 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C40">
@@ -912,7 +912,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C41">
@@ -925,7 +925,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">3 × 1,470 m (Izq) + 1 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C42">
@@ -1068,11 +1068,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,470 m (Fondo) + 1 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C53">
-        <v>0.18</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="54">
@@ -1081,11 +1081,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C54">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="55">
@@ -1094,11 +1094,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,470 m (Fondo) + 1 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C55">
-        <v>0.39</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="56">
@@ -1159,11 +1159,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,400 m (Puerta) + 2 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C60">
-        <v>0.01</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="61">
@@ -1172,10 +1172,36 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C61">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <v>60</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,400 m (Puerta) + 2 × 0,888 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C62">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <v>61</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
           <t xml:space="preserve">1 × 0,888 m (Puerta)</t>
         </is>
       </c>
-      <c r="C61">
+      <c r="C63">
         <v>5.11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fachada La Carreta: frente de 8 m con 3 pilares y decorado mas parecido a la foto
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DFEggjd6XpHEYcqFvcrgyh
</commit_message>
<xml_diff>
--- a/fachada-la-carreta/lista-materiales-fachada-la-carreta.xlsx
+++ b/fachada-la-carreta/lista-materiales-fachada-la-carreta.xlsx
@@ -69,7 +69,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Frente 4,00 m · Alto 3,00 m · Fondo 4,00 m · Tubo 20×20 mm</t>
+          <t xml:space="preserve">Frente 8,00 m · Alto 3,00 m · Fondo 4,00 m · Tubo 20×20 mm</t>
         </is>
       </c>
     </row>
@@ -103,7 +103,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>61</v>
+        <v>91</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -112,7 +112,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">sobrante 13,02 m</t>
+          <t xml:space="preserve">sobrante 18,51 m</t>
         </is>
       </c>
     </row>
@@ -268,7 +268,7 @@
         </is>
       </c>
       <c r="B14">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -277,7 +277,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">24 en paneles + 8 bajo los rieles</t>
+          <t xml:space="preserve">32 en paneles + 8 bajo los rieles</t>
         </is>
       </c>
     </row>
@@ -288,7 +288,7 @@
         </is>
       </c>
       <c r="B15">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -308,7 +308,7 @@
         </is>
       </c>
       <c r="B16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -317,7 +317,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Área de tubo: 28,2 m², una mano</t>
+          <t xml:space="preserve">Área de tubo: 42,1 m², una mano</t>
         </is>
       </c>
     </row>
@@ -328,7 +328,7 @@
         </is>
       </c>
       <c r="B17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -348,7 +348,7 @@
         </is>
       </c>
       <c r="B18">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -357,7 +357,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mi cálculo para 466 uniones soldadas. Con las medidas anteriores usaste 3 lb</t>
+          <t xml:space="preserve">Mi cálculo para 686 uniones soldadas. Con las medidas anteriores usaste 3 lb</t>
         </is>
       </c>
     </row>
@@ -418,7 +418,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fijo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C3">
@@ -431,7 +431,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fijo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C4">
@@ -444,7 +444,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fijo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C5">
@@ -457,7 +457,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C6">
@@ -470,7 +470,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C7">
@@ -483,7 +483,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C8">
@@ -496,7 +496,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">1 × 3,550 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C9">
@@ -509,7 +509,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">1 × 3,550 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C10">
@@ -522,7 +522,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">1 × 3,550 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C11">
@@ -535,11 +535,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C12">
-        <v>0.11</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="13">
@@ -548,11 +548,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C13">
-        <v>0.11</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="14">
@@ -561,11 +561,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C14">
-        <v>0.11</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="15">
@@ -574,11 +574,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C15">
-        <v>0.11</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="16">
@@ -587,11 +587,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,470 m (Fijo) + 1 × 1,470 m (Der)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C16">
-        <v>0.11</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="17">
@@ -600,11 +600,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C17">
-        <v>0.11</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="18">
@@ -613,7 +613,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C18">
@@ -626,7 +626,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C19">
@@ -639,7 +639,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C20">
@@ -652,7 +652,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C21">
@@ -665,7 +665,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C22">
@@ -678,7 +678,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C23">
@@ -691,7 +691,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C24">
@@ -704,7 +704,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C25">
@@ -717,7 +717,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C26">
@@ -730,7 +730,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C27">
@@ -743,7 +743,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C28">
@@ -756,7 +756,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,470 m (Der) + 1 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C29">
@@ -769,7 +769,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C30">
@@ -782,7 +782,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C31">
@@ -795,7 +795,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C32">
@@ -808,7 +808,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C33">
@@ -821,7 +821,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">1 × 1,470 m (Fijo) + 3 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C34">
@@ -834,7 +834,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C35">
@@ -847,7 +847,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C36">
@@ -860,7 +860,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C37">
@@ -873,7 +873,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C38">
@@ -886,7 +886,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C39">
@@ -899,7 +899,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C40">
@@ -912,7 +912,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C41">
@@ -925,7 +925,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,470 m (Izq) + 1 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C42">
@@ -938,7 +938,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C43">
@@ -951,7 +951,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C44">
@@ -964,7 +964,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C45">
@@ -977,7 +977,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C46">
@@ -990,7 +990,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">1 × 1,470 m (Der) + 3 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C47">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C48">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C49">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C50">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C51">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C52">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C53">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C54">
@@ -1094,11 +1094,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,470 m (Fondo) + 1 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C55">
-        <v>0.18</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="56">
@@ -1107,11 +1107,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C56">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="57">
@@ -1120,11 +1120,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C57">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="58">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C58">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="59">
@@ -1146,11 +1146,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C59">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="60">
@@ -1159,11 +1159,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">1 × 1,470 m (Izq) + 3 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C60">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="61">
@@ -1172,11 +1172,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C61">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="62">
@@ -1185,11 +1185,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,400 m (Puerta) + 2 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C62">
-        <v>0.01</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="63">
@@ -1198,11 +1198,401 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C63">
-        <v>5.11</v>
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64">
+        <v>62</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C64">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65">
+        <v>63</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C65">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66">
+        <v>64</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C66">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67">
+        <v>65</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C67">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68">
+        <v>66</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C68">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69">
+        <v>67</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C69">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70">
+        <v>68</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C70">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71">
+        <v>69</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C71">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72">
+        <v>70</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C72">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73">
+        <v>71</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C73">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74">
+        <v>72</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C74">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75">
+        <v>73</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C75">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76">
+        <v>74</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C76">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77">
+        <v>75</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C77">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78">
+        <v>76</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C78">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79">
+        <v>77</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C79">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80">
+        <v>78</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C80">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81">
+        <v>79</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C81">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82">
+        <v>80</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C82">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83">
+        <v>81</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C83">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84">
+        <v>82</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C84">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85">
+        <v>83</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C85">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86">
+        <v>84</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 × 1,470 m (Fondo) + 3 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C86">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87">
+        <v>85</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C87">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88">
+        <v>86</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C88">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89">
+        <v>87</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C89">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90">
+        <v>88</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C90">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91">
+        <v>89</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C91">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92">
+        <v>90</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C92">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93">
+        <v>91</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C93">
+        <v>4.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fachada La Carreta: 2 puertas corredizas en un solo lugar y opciones de puerta claras
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DFEggjd6XpHEYcqFvcrgyh
</commit_message>
<xml_diff>
--- a/fachada-la-carreta/lista-materiales-fachada-la-carreta.xlsx
+++ b/fachada-la-carreta/lista-materiales-fachada-la-carreta.xlsx
@@ -172,7 +172,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 por puerta</t>
+          <t xml:space="preserve">2 por cada una de las 2 puertas</t>
         </is>
       </c>
     </row>
@@ -192,7 +192,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 por puerta</t>
+          <t xml:space="preserve">2 por cada una de las 2 puertas</t>
         </is>
       </c>
     </row>
@@ -258,6 +258,11 @@
       <c r="C13" t="inlineStr">
         <is>
           <t xml:space="preserve">u</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Una por puerta</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fachada La Carreta: una puerta corrediza en cada tramo del frente
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DFEggjd6XpHEYcqFvcrgyh
</commit_message>
<xml_diff>
--- a/fachada-la-carreta/lista-materiales-fachada-la-carreta.xlsx
+++ b/fachada-la-carreta/lista-materiales-fachada-la-carreta.xlsx
@@ -112,7 +112,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">sobrante 18,51 m</t>
+          <t xml:space="preserve">sobrante 14,55 m</t>
         </is>
       </c>
     </row>
@@ -123,7 +123,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -143,7 +143,7 @@
         </is>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -163,7 +163,7 @@
         </is>
       </c>
       <c r="B8">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -172,7 +172,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 por cada una de las 2 puertas</t>
+          <t xml:space="preserve">4 por puerta (2 por hoja)</t>
         </is>
       </c>
     </row>
@@ -183,7 +183,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -192,7 +192,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 por cada una de las 2 puertas</t>
+          <t xml:space="preserve">4 por puerta (2 por hoja)</t>
         </is>
       </c>
     </row>
@@ -203,7 +203,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -218,7 +218,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -233,7 +233,7 @@
         </is>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -253,7 +253,7 @@
         </is>
       </c>
       <c r="B13">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -262,7 +262,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Una por puerta</t>
+          <t xml:space="preserve">Una por hoja (2 hojas por puerta)</t>
         </is>
       </c>
     </row>
@@ -273,7 +273,7 @@
         </is>
       </c>
       <c r="B14">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -282,7 +282,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">32 en paneles + 8 bajo los rieles</t>
+          <t xml:space="preserve">32 en paneles + 16 bajo los rieles</t>
         </is>
       </c>
     </row>
@@ -293,7 +293,7 @@
         </is>
       </c>
       <c r="B15">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -322,7 +322,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Área de tubo: 42,1 m², una mano</t>
+          <t xml:space="preserve">Área de tubo: 42,4 m², una mano</t>
         </is>
       </c>
     </row>
@@ -362,7 +362,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mi cálculo para 686 uniones soldadas. Con las medidas anteriores usaste 3 lb</t>
+          <t xml:space="preserve">Mi cálculo para 712 uniones soldadas. Con las medidas anteriores usaste 3 lb</t>
         </is>
       </c>
     </row>
@@ -423,7 +423,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fijo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C3">
@@ -436,7 +436,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fijo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C4">
@@ -449,7 +449,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fijo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C5">
@@ -462,7 +462,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C6">
@@ -475,7 +475,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C7">
@@ -488,7 +488,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C8">
@@ -501,7 +501,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C9">
@@ -514,7 +514,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C10">
@@ -527,7 +527,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C11">
@@ -540,7 +540,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C12">
@@ -553,7 +553,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C13">
@@ -566,7 +566,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C14">
@@ -579,11 +579,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C15">
-        <v>0.97</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="16">
@@ -592,11 +592,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C16">
-        <v>0.97</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="17">
@@ -605,11 +605,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C17">
-        <v>0.97</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="18">
@@ -722,7 +722,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C26">
@@ -735,7 +735,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C27">
@@ -748,7 +748,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C28">
@@ -761,7 +761,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C29">
@@ -774,7 +774,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C30">
@@ -787,7 +787,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C31">
@@ -800,7 +800,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C32">
@@ -813,7 +813,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C33">
@@ -826,7 +826,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 1,470 m (Fijo) + 3 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C34">
@@ -891,7 +891,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C39">
@@ -904,7 +904,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C40">
@@ -917,7 +917,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C41">
@@ -930,7 +930,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C42">
@@ -943,7 +943,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C43">
@@ -956,7 +956,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C44">
@@ -969,7 +969,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C45">
@@ -982,7 +982,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C46">
@@ -995,7 +995,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 1,470 m (Der) + 3 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C47">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C52">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C53">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C54">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C55">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C56">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C57">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C58">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C59">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 1,470 m (Izq) + 3 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C60">
@@ -1398,11 +1398,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C78">
-        <v>0.11</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="79">
@@ -1411,11 +1411,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C79">
-        <v>0.11</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="80">
@@ -1424,11 +1424,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C80">
-        <v>0.11</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="81">
@@ -1437,11 +1437,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C81">
-        <v>0.11</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="82">
@@ -1450,11 +1450,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C82">
-        <v>0.11</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="83">
@@ -1463,11 +1463,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C83">
-        <v>0.11</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="84">
@@ -1476,11 +1476,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C84">
-        <v>0.11</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="85">
@@ -1489,11 +1489,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C85">
-        <v>0.11</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="86">
@@ -1502,11 +1502,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 1,470 m (Fondo) + 3 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C86">
-        <v>0.32</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="87">
@@ -1580,11 +1580,11 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">6 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C92">
-        <v>0.39</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="93">
@@ -1593,11 +1593,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">6 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C93">
-        <v>4.6</v>
+        <v>0.66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fachada La Carreta: pilares delgados de metal en costados y fondo, 3 por costado
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DFEggjd6XpHEYcqFvcrgyh
</commit_message>
<xml_diff>
--- a/fachada-la-carreta/lista-materiales-fachada-la-carreta.xlsx
+++ b/fachada-la-carreta/lista-materiales-fachada-la-carreta.xlsx
@@ -103,7 +103,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -112,7 +112,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">sobrante 14,55 m</t>
+          <t xml:space="preserve">sobrante 18,61 m</t>
         </is>
       </c>
     </row>
@@ -273,7 +273,7 @@
         </is>
       </c>
       <c r="B14">
-        <v>48</v>
+        <v>72</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -282,7 +282,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">32 en paneles + 16 bajo los rieles</t>
+          <t xml:space="preserve">56 en paneles + 16 bajo los rieles</t>
         </is>
       </c>
     </row>
@@ -293,7 +293,7 @@
         </is>
       </c>
       <c r="B15">
-        <v>96</v>
+        <v>144</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -322,7 +322,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Área de tubo: 42,4 m², una mano</t>
+          <t xml:space="preserve">Área de tubo: 44,0 m², una mano</t>
         </is>
       </c>
     </row>
@@ -362,7 +362,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mi cálculo para 712 uniones soldadas. Con las medidas anteriores usaste 3 lb</t>
+          <t xml:space="preserve">Mi cálculo para 748 uniones soldadas. Con las medidas anteriores usaste 3 lb</t>
         </is>
       </c>
     </row>
@@ -423,11 +423,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,880 m (Der)</t>
         </is>
       </c>
       <c r="C3">
-        <v>0.08</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="4">
@@ -436,11 +436,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,880 m (Der)</t>
         </is>
       </c>
       <c r="C4">
-        <v>0.08</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="5">
@@ -449,11 +449,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,880 m (Der)</t>
         </is>
       </c>
       <c r="C5">
-        <v>0.08</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="6">
@@ -462,11 +462,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,880 m (Izq)</t>
         </is>
       </c>
       <c r="C6">
-        <v>0.08</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="7">
@@ -475,11 +475,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,880 m (Izq)</t>
         </is>
       </c>
       <c r="C7">
-        <v>0.08</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="8">
@@ -488,11 +488,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,880 m (Izq)</t>
         </is>
       </c>
       <c r="C8">
-        <v>0.08</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="9">
@@ -501,11 +501,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">3 × 1,715 m (Der)</t>
         </is>
       </c>
       <c r="C9">
-        <v>0.08</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="10">
@@ -514,11 +514,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">3 × 1,715 m (Izq)</t>
         </is>
       </c>
       <c r="C10">
-        <v>0.08</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="11">
@@ -527,11 +527,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C11">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="12">
@@ -540,11 +540,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C12">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="13">
@@ -553,11 +553,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C13">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="14">
@@ -566,11 +566,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C14">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="15">
@@ -709,7 +709,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C25">
@@ -878,7 +878,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">2 × 1,470 m (Der) + 2 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C38">
@@ -1398,11 +1398,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C78">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="79">
@@ -1411,11 +1411,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C79">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="80">
@@ -1580,11 +1580,11 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C92">
-        <v>0.66</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="93">
@@ -1593,10 +1593,62 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C93">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94">
+        <v>92</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 × 0,888 m (Fijo)</t>
+        </is>
+      </c>
+      <c r="C94">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95">
+        <v>93</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 × 0,888 m (Fijo)</t>
+        </is>
+      </c>
+      <c r="C95">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96">
+        <v>94</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
           <t xml:space="preserve">6 × 0,888 m (Puerta)</t>
         </is>
       </c>
-      <c r="C93">
+      <c r="C96">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97">
+        <v>95</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 × 0,888 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C97">
         <v>0.66</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fachada La Carreta: fondo de 8 m, 2 tramos fijos por lado como el frente
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DFEggjd6XpHEYcqFvcrgyh
</commit_message>
<xml_diff>
--- a/fachada-la-carreta/lista-materiales-fachada-la-carreta.xlsx
+++ b/fachada-la-carreta/lista-materiales-fachada-la-carreta.xlsx
@@ -69,7 +69,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Frente 8,00 m · Alto 3,00 m · Fondo 4,00 m · Tubo 20×20 mm</t>
+          <t xml:space="preserve">Frente 8,00 m · Alto 3,00 m · Fondo 8,00 m · Tubo 20×20 mm</t>
         </is>
       </c>
     </row>
@@ -103,7 +103,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>95</v>
+        <v>129</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -112,7 +112,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">sobrante 18,61 m</t>
+          <t xml:space="preserve">sobrante 33,63 m</t>
         </is>
       </c>
     </row>
@@ -273,7 +273,7 @@
         </is>
       </c>
       <c r="B14">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -282,7 +282,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">56 en paneles + 16 bajo los rieles</t>
+          <t xml:space="preserve">64 en paneles + 16 bajo los rieles</t>
         </is>
       </c>
     </row>
@@ -293,7 +293,7 @@
         </is>
       </c>
       <c r="B15">
-        <v>144</v>
+        <v>160</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -322,7 +322,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Área de tubo: 44,0 m², una mano</t>
+          <t xml:space="preserve">Área de tubo: 59,1 m², una mano</t>
         </is>
       </c>
     </row>
@@ -333,7 +333,7 @@
         </is>
       </c>
       <c r="B17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -353,7 +353,7 @@
         </is>
       </c>
       <c r="B18">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -362,7 +362,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mi cálculo para 748 uniones soldadas. Con las medidas anteriores usaste 3 lb</t>
+          <t xml:space="preserve">Mi cálculo para 972 uniones soldadas. Con las medidas anteriores usaste 3 lb</t>
         </is>
       </c>
     </row>
@@ -423,11 +423,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,880 m (Der)</t>
+          <t xml:space="preserve">1 × 3,880 m (Der) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C3">
-        <v>0.23</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="4">
@@ -436,11 +436,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,880 m (Der)</t>
+          <t xml:space="preserve">1 × 3,880 m (Der) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C4">
-        <v>0.23</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="5">
@@ -449,11 +449,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,880 m (Der)</t>
+          <t xml:space="preserve">1 × 3,880 m (Der) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C5">
-        <v>0.23</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="6">
@@ -462,11 +462,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,880 m (Izq)</t>
+          <t xml:space="preserve">1 × 3,880 m (Izq) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C6">
-        <v>0.23</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="7">
@@ -475,11 +475,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,880 m (Izq)</t>
+          <t xml:space="preserve">1 × 3,880 m (Izq) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C7">
-        <v>0.23</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="8">
@@ -488,11 +488,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,880 m (Izq)</t>
+          <t xml:space="preserve">1 × 3,880 m (Izq) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C8">
-        <v>0.23</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="9">
@@ -501,11 +501,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,715 m (Der)</t>
+          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C9">
-        <v>0.85</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="10">
@@ -514,11 +514,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,715 m (Izq)</t>
+          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C10">
-        <v>0.85</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="11">
@@ -527,11 +527,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C11">
-        <v>0.11</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="12">
@@ -540,11 +540,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C12">
-        <v>0.11</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="13">
@@ -553,11 +553,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C13">
-        <v>0.11</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="14">
@@ -566,11 +566,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C14">
-        <v>0.11</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="15">
@@ -579,11 +579,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,715 m (Der) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C15">
-        <v>0.11</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="16">
@@ -592,11 +592,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,715 m (Der) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C16">
-        <v>0.11</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="17">
@@ -605,11 +605,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,715 m (Der) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C17">
-        <v>0.11</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="18">
@@ -618,11 +618,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,715 m (Izq) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C18">
-        <v>0.11</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="19">
@@ -631,11 +631,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,715 m (Izq) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C19">
-        <v>0.11</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="20">
@@ -644,11 +644,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,715 m (Izq) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C20">
-        <v>0.11</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="21">
@@ -709,7 +709,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C25">
@@ -722,7 +722,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C26">
@@ -735,7 +735,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C27">
@@ -748,7 +748,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C28">
@@ -761,7 +761,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C29">
@@ -774,7 +774,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Der)</t>
+          <t xml:space="preserve">2 × 1,470 m (Fijo) + 2 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C30">
@@ -878,7 +878,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 × 1,470 m (Der) + 2 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C38">
@@ -891,7 +891,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C39">
@@ -904,7 +904,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C40">
@@ -917,7 +917,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C41">
@@ -930,7 +930,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C42">
@@ -943,7 +943,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C43">
@@ -956,7 +956,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C44">
@@ -969,7 +969,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C45">
@@ -982,7 +982,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C46">
@@ -995,7 +995,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C47">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C48">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C49">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C50">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C51">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C52">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C53">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C54">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C55">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C56">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C57">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C58">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C59">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C60">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C61">
@@ -1190,7 +1190,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C62">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C63">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C64">
@@ -1229,7 +1229,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C65">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C66">
@@ -1255,7 +1255,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C67">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C68">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C69">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C70">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C71">
@@ -1320,7 +1320,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C72">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C73">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C74">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C75">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C76">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C77">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C78">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C79">
@@ -1424,11 +1424,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C80">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="81">
@@ -1437,11 +1437,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C81">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="82">
@@ -1450,11 +1450,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C82">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="83">
@@ -1463,11 +1463,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C83">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="84">
@@ -1476,11 +1476,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C84">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="85">
@@ -1489,11 +1489,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">2 × 1,470 m (Izq) + 2 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C85">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="86">
@@ -1502,11 +1502,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C86">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="87">
@@ -1515,11 +1515,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C87">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="88">
@@ -1528,11 +1528,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C88">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="89">
@@ -1541,11 +1541,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C89">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="90">
@@ -1554,11 +1554,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C90">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="91">
@@ -1567,11 +1567,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C91">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="92">
@@ -1580,11 +1580,11 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C92">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="93">
@@ -1593,11 +1593,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C93">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="94">
@@ -1606,11 +1606,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C94">
-        <v>0.66</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="95">
@@ -1619,11 +1619,11 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C95">
-        <v>0.66</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="96">
@@ -1632,11 +1632,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C96">
-        <v>0.66</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="97">
@@ -1645,11 +1645,453 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C97">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98">
+        <v>96</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C98">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99">
+        <v>97</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C99">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100">
+        <v>98</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C100">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101">
+        <v>99</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C101">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102">
+        <v>100</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C102">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103">
+        <v>101</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C103">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104">
+        <v>102</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C104">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105">
+        <v>103</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C105">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106">
+        <v>104</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C106">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107">
+        <v>105</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C107">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108">
+        <v>106</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C108">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109">
+        <v>107</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C109">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110">
+        <v>108</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C110">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111">
+        <v>109</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C111">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112">
+        <v>110</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C112">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113">
+        <v>111</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 × 1,470 m (Fondo) + 2 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C113">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114">
+        <v>112</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C114">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115">
+        <v>113</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C115">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116">
+        <v>114</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C116">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117">
+        <v>115</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C117">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118">
+        <v>116</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C118">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119">
+        <v>117</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C119">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120">
+        <v>118</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C120">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121">
+        <v>119</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C121">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122">
+        <v>120</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C122">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123">
+        <v>121</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C123">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124">
+        <v>122</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C124">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125">
+        <v>123</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C125">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126">
+        <v>124</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C126">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127">
+        <v>125</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 × 1,400 m (Puerta) + 3 × 0,888 m (Fijo)</t>
+        </is>
+      </c>
+      <c r="C127">
+        <v>0.52</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128">
+        <v>126</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 × 0,888 m (Fijo)</t>
+        </is>
+      </c>
+      <c r="C128">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129">
+        <v>127</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 0,888 m (Fijo) + 3 × 0,888 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C129">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130">
+        <v>128</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
           <t xml:space="preserve">6 × 0,888 m (Puerta)</t>
         </is>
       </c>
-      <c r="C97">
+      <c r="C130">
         <v>0.66</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131">
+        <v>129</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 0,888 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C131">
+        <v>3.33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fachada La Carreta: pared trasera con 2 tramos visibles (pilar ancho al medio)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DFEggjd6XpHEYcqFvcrgyh
</commit_message>
<xml_diff>
--- a/fachada-la-carreta/lista-materiales-fachada-la-carreta.xlsx
+++ b/fachada-la-carreta/lista-materiales-fachada-la-carreta.xlsx
@@ -103,7 +103,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -112,7 +112,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">sobrante 33,63 m</t>
+          <t xml:space="preserve">sobrante 34,51 m</t>
         </is>
       </c>
     </row>
@@ -322,7 +322,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Área de tubo: 59,1 m², una mano</t>
+          <t xml:space="preserve">Área de tubo: 58,6 m², una mano</t>
         </is>
       </c>
     </row>
@@ -362,7 +362,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mi cálculo para 972 uniones soldadas. Con las medidas anteriores usaste 3 lb</t>
+          <t xml:space="preserve">Mi cálculo para 964 uniones soldadas. Con las medidas anteriores usaste 3 lb</t>
         </is>
       </c>
     </row>
@@ -501,11 +501,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,715 m (Der) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C9">
-        <v>0.64</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="10">
@@ -514,11 +514,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,715 m (Der) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C10">
-        <v>0.64</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="11">
@@ -527,11 +527,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,715 m (Der) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C11">
-        <v>0.64</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="12">
@@ -540,11 +540,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,715 m (Izq) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C12">
-        <v>0.64</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="13">
@@ -553,11 +553,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,715 m (Izq) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C13">
-        <v>0.64</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="14">
@@ -566,11 +566,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,880 m (Fondo) + 1 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,715 m (Izq) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C14">
-        <v>0.64</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="15">
@@ -579,7 +579,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,715 m (Der) + 1 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,715 m (Fondo) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C15">
@@ -592,7 +592,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,715 m (Der) + 1 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,715 m (Fondo) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C16">
@@ -605,7 +605,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,715 m (Der) + 1 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,715 m (Fondo) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C17">
@@ -618,7 +618,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,715 m (Izq) + 1 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,715 m (Fondo) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C18">
@@ -631,7 +631,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,715 m (Izq) + 1 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,715 m (Fondo) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C19">
@@ -644,7 +644,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,715 m (Izq) + 1 × 1,470 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,715 m (Fondo) + 1 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C20">
@@ -1840,11 +1840,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
+          <t xml:space="preserve">2 × 1,470 m (Fondo) + 2 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C112">
-        <v>0.11</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="113">
@@ -1853,11 +1853,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 × 1,470 m (Fondo) + 2 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C113">
-        <v>0.25</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="114">
@@ -2022,11 +2022,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
+          <t xml:space="preserve">2 × 1,400 m (Puerta) + 3 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C126">
-        <v>0.39</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="127">
@@ -2035,11 +2035,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 × 1,400 m (Puerta) + 3 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">6 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C127">
-        <v>0.52</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="128">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">3 × 0,888 m (Fijo) + 3 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C128">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 0,888 m (Fijo) + 3 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">6 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C129">
@@ -2074,23 +2074,10 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">3 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C130">
-        <v>0.66</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131">
-        <v>129</v>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 × 0,888 m (Puerta)</t>
-        </is>
-      </c>
-      <c r="C131">
         <v>3.33</v>
       </c>
     </row>

</xml_diff>